<commit_message>
wip: e2e, docs and finals note
</commit_message>
<xml_diff>
--- a/academy/src/finals/Q3_Commercial_Final.xlsx
+++ b/academy/src/finals/Q3_Commercial_Final.xlsx
@@ -1243,11 +1243,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="75825592"/>
-        <c:axId val="68291026"/>
+        <c:axId val="39525077"/>
+        <c:axId val="40855803"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="75825592"/>
+        <c:axId val="39525077"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1275,7 +1275,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68291026"/>
+        <c:crossAx val="40855803"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1283,7 +1283,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="68291026"/>
+        <c:axId val="40855803"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1321,7 +1321,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75825592"/>
+        <c:crossAx val="39525077"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1498,11 +1498,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="66704419"/>
-        <c:axId val="39342873"/>
+        <c:axId val="75901053"/>
+        <c:axId val="6949632"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="66704419"/>
+        <c:axId val="75901053"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1530,7 +1530,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39342873"/>
+        <c:crossAx val="6949632"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1538,7 +1538,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="39342873"/>
+        <c:axId val="6949632"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1576,7 +1576,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66704419"/>
+        <c:crossAx val="75901053"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1764,11 +1764,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="42793920"/>
-        <c:axId val="16469210"/>
+        <c:axId val="70169100"/>
+        <c:axId val="9355037"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="42793920"/>
+        <c:axId val="70169100"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1796,7 +1796,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16469210"/>
+        <c:crossAx val="9355037"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1804,7 +1804,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="16469210"/>
+        <c:axId val="9355037"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1842,7 +1842,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42793920"/>
+        <c:crossAx val="70169100"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2000,11 +2000,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="86264801"/>
-        <c:axId val="16515245"/>
+        <c:axId val="51347692"/>
+        <c:axId val="69499584"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86264801"/>
+        <c:axId val="51347692"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2032,7 +2032,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16515245"/>
+        <c:crossAx val="69499584"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2040,7 +2040,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="16515245"/>
+        <c:axId val="69499584"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2078,7 +2078,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86264801"/>
+        <c:crossAx val="51347692"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Finished dashboard reads the pivot tables, so slicers filter its figures and charts
The example-1 dashboard's KPIs use GETPIVOTDATA and its four charts read a chart-data
block filled from the pivot tables, instead of the full-quarter Report sheet. A data
test checks the dashboard formulas and chart references (review finding on PR 41).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CHMU38Chok4mRKjeuEBFA6
</commit_message>
<xml_diff>
--- a/academy/src/finals/Q3_Commercial_Final.xlsx
+++ b/academy/src/finals/Q3_Commercial_Final.xlsx
@@ -1243,11 +1243,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="39525077"/>
-        <c:axId val="40855803"/>
+        <c:axId val="17139343"/>
+        <c:axId val="38136934"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="39525077"/>
+        <c:axId val="17139343"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1275,7 +1275,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40855803"/>
+        <c:crossAx val="38136934"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1283,7 +1283,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40855803"/>
+        <c:axId val="38136934"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1321,7 +1321,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39525077"/>
+        <c:crossAx val="17139343"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1498,11 +1498,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="75901053"/>
-        <c:axId val="6949632"/>
+        <c:axId val="65121689"/>
+        <c:axId val="52760127"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="75901053"/>
+        <c:axId val="65121689"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1530,7 +1530,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6949632"/>
+        <c:crossAx val="52760127"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1538,7 +1538,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6949632"/>
+        <c:axId val="52760127"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1576,7 +1576,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75901053"/>
+        <c:crossAx val="65121689"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1764,11 +1764,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="70169100"/>
-        <c:axId val="9355037"/>
+        <c:axId val="95515358"/>
+        <c:axId val="58935922"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="70169100"/>
+        <c:axId val="95515358"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1796,7 +1796,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9355037"/>
+        <c:crossAx val="58935922"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1804,7 +1804,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9355037"/>
+        <c:axId val="58935922"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1842,7 +1842,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70169100"/>
+        <c:crossAx val="95515358"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2000,11 +2000,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="51347692"/>
-        <c:axId val="69499584"/>
+        <c:axId val="81334836"/>
+        <c:axId val="66055054"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="51347692"/>
+        <c:axId val="81334836"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2032,7 +2032,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69499584"/>
+        <c:crossAx val="66055054"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2040,7 +2040,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69499584"/>
+        <c:axId val="66055054"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2078,7 +2078,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51347692"/>
+        <c:crossAx val="81334836"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>